<commit_message>
Rectified issues in statistical analysis
</commit_message>
<xml_diff>
--- a/analysis/results/statistical_analysis.xlsx
+++ b/analysis/results/statistical_analysis.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Descriptive Statistics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Friedman Test" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pairwise Comparisons" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Average Ranks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1582,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1598,37 +1598,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Raw p-value</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Holm-adjusted p-value</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Significant</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Effect size</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Effect size method</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>N effective</t>
+          <t>Average Rank</t>
         </is>
       </c>
     </row>
@@ -1645,28 +1620,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1686,24 +1644,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="4">
@@ -1723,24 +1664,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="5">
@@ -1756,28 +1680,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="6">
@@ -1793,28 +1700,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>5</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="7">
@@ -1825,7 +1715,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>mape</t>
+          <t>mae</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1834,24 +1724,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -1867,28 +1740,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
         <v>1</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1904,28 +1760,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>cnn</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="10">
@@ -1941,28 +1780,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F10" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="11">
@@ -1978,28 +1800,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.4375</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.4375</v>
-      </c>
-      <c r="F11" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.4666666666666667</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -2010,33 +1815,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F12" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="13">
@@ -2047,33 +1835,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F13" t="b">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="14">
@@ -2089,28 +1860,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2126,28 +1880,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F15" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="16">
@@ -2163,28 +1900,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F16" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="17">
@@ -2195,33 +1915,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F17" t="b">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="18">
@@ -2232,32 +1935,15 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F18" t="b">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2269,33 +1955,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>cnn</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F19" t="b">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -2311,28 +1980,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
         <v>1</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -2348,28 +2000,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F21" t="b">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="22">
@@ -2380,33 +2015,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F22" t="b">
-        <v>0</v>
-      </c>
-      <c r="G22" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="23">
@@ -2417,33 +2035,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F23" t="b">
-        <v>0</v>
-      </c>
-      <c r="G23" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="24">
@@ -2454,32 +2055,15 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F24" t="b">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2491,33 +2075,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>cnn</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F25" t="b">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -2533,28 +2100,111 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>dcnn_rbilstm</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>lstm</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
           <t>proposed_no_ta</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F26" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>rank_biserial</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>5</v>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>cnn</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated statistical analysis based on all models including ablation ones
</commit_message>
<xml_diff>
--- a/analysis/results/statistical_analysis.xlsx
+++ b/analysis/results/statistical_analysis.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,24 +596,24 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4.184532451629638</v>
+        <v>4.216937065124512</v>
       </c>
       <c r="E6" t="n">
-        <v>0.08878983524430208</v>
+        <v>0.08402373730557748</v>
       </c>
       <c r="F6" t="n">
         <v>5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4.185 ± 0.08879</t>
+          <t>4.217 ± 0.08402</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>proposed_no_fa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -627,24 +627,24 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4.527873516082764</v>
+        <v>4.207920360565185</v>
       </c>
       <c r="E7" t="n">
-        <v>0.06594824943905804</v>
+        <v>0.05102146108293532</v>
       </c>
       <c r="F7" t="n">
         <v>5</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4.528 ± 0.06595</t>
+          <t>4.208 ± 0.05102</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>proposed_no_fusion</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -654,28 +654,28 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>mape</t>
+          <t>mae</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4725856.6</v>
+        <v>4.259976482391357</v>
       </c>
       <c r="E8" t="n">
-        <v>28187.48356629233</v>
+        <v>0.0680074523312066</v>
       </c>
       <c r="F8" t="n">
         <v>5</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4.726e+06 ± 2.819e+04</t>
+          <t>4.26 ± 0.06801</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -685,28 +685,28 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>mape</t>
+          <t>mae</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4726949.8</v>
+        <v>4.527873516082764</v>
       </c>
       <c r="E9" t="n">
-        <v>16888.35301546601</v>
+        <v>0.06594824943905804</v>
       </c>
       <c r="F9" t="n">
         <v>5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4.727e+06 ± 1.689e+04</t>
+          <t>4.528 ± 0.06595</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>cnn</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -720,24 +720,24 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4769878.7</v>
+        <v>4725856.6</v>
       </c>
       <c r="E10" t="n">
-        <v>18520.94431515305</v>
+        <v>28187.48356629233</v>
       </c>
       <c r="F10" t="n">
         <v>5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4.77e+06 ± 1.852e+04</t>
+          <t>4.726e+06 ± 2.819e+04</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -751,24 +751,24 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4841693.2</v>
+        <v>4726949.8</v>
       </c>
       <c r="E11" t="n">
-        <v>28615.53728440198</v>
+        <v>16888.35301546601</v>
       </c>
       <c r="F11" t="n">
         <v>5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4.842e+06 ± 2.862e+04</t>
+          <t>4.727e+06 ± 1.689e+04</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -782,24 +782,24 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>4883865.8</v>
+        <v>4769878.7</v>
       </c>
       <c r="E12" t="n">
-        <v>64790.83971866702</v>
+        <v>18520.94431515305</v>
       </c>
       <c r="F12" t="n">
         <v>5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4.884e+06 ± 6.479e+04</t>
+          <t>4.77e+06 ± 1.852e+04</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -813,24 +813,24 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4664677.3</v>
+        <v>4841693.2</v>
       </c>
       <c r="E13" t="n">
-        <v>31127.43013725997</v>
+        <v>28615.53728440198</v>
       </c>
       <c r="F13" t="n">
         <v>5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4.665e+06 ± 3.113e+04</t>
+          <t>4.842e+06 ± 2.862e+04</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -840,28 +840,28 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.04979401603036462</v>
+        <v>3984548.44375</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0003048641542901735</v>
+        <v>2003245.536608462</v>
       </c>
       <c r="F14" t="n">
         <v>5</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.04979 ± 0.0003049</t>
+          <t>3.985e+06 ± 2.003e+06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed_no_fa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -871,28 +871,28 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.04855114754415745</v>
+        <v>401800.075</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0002775955214901212</v>
+        <v>3842.078874887835</v>
       </c>
       <c r="F15" t="n">
         <v>5</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.04855 ± 0.0002776</t>
+          <t>4.018e+05 ± 3842</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed_no_fusion</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -902,28 +902,28 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.04846874226264738</v>
+        <v>398547.6875</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0002280812613149944</v>
+        <v>4175.73194206155</v>
       </c>
       <c r="F16" t="n">
         <v>5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0.04847 ± 0.0002281</t>
+          <t>3.985e+05 ± 4176</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -933,28 +933,28 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.04878313843667011</v>
+        <v>4664677.3</v>
       </c>
       <c r="E17" t="n">
-        <v>0.00015545824115454</v>
+        <v>31127.43013725997</v>
       </c>
       <c r="F17" t="n">
         <v>5</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>0.04878 ± 0.0001555</t>
+          <t>4.665e+06 ± 3.113e+04</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>cnn</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -968,24 +968,24 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.04787772880144144</v>
+        <v>0.04979401603036462</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0002142692118711192</v>
+        <v>0.0003048641542901735</v>
       </c>
       <c r="F18" t="n">
         <v>5</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.04788 ± 0.0002143</t>
+          <t>0.04979 ± 0.0003049</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -999,24 +999,24 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.0492212808790379</v>
+        <v>0.04855114754415745</v>
       </c>
       <c r="E19" t="n">
-        <v>0.000275921959119208</v>
+        <v>0.0002775955214901212</v>
       </c>
       <c r="F19" t="n">
         <v>5</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0.04922 ± 0.0002759</t>
+          <t>0.04855 ± 0.0002776</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1026,28 +1026,28 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.9673994421958924</v>
+        <v>0.04846874226264738</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0003991396556738538</v>
+        <v>0.0002280812613149944</v>
       </c>
       <c r="F20" t="n">
         <v>5</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.9674 ± 0.0003991</t>
+          <t>0.04847 ± 0.0002281</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1057,28 +1057,28 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.9690066933631897</v>
+        <v>0.04878313843667011</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0003546163641341093</v>
+        <v>0.00015545824115454</v>
       </c>
       <c r="F21" t="n">
         <v>5</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.969 ± 0.0003546</t>
+          <t>0.04878 ± 0.0001555</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1088,28 +1088,28 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.9691120862960816</v>
+        <v>0.04798688366446857</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0002913077525296171</v>
+        <v>0.0003110358287359922</v>
       </c>
       <c r="F22" t="n">
         <v>5</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0.9691 ± 0.0002913</t>
+          <t>0.04799 ± 0.000311</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>proposed_no_fa</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1119,28 +1119,28 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.9687103509902955</v>
+        <v>0.04820234160450318</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0001997038942132785</v>
+        <v>0.0002735703066835043</v>
       </c>
       <c r="F23" t="n">
         <v>5</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.9687 ± 0.0001997</t>
+          <t>0.0482 ± 0.0002736</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>proposed_no_fusion</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1150,21 +1150,21 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.9698608040809631</v>
+        <v>0.04810661408588918</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0002699098242906955</v>
+        <v>0.0001918931528414719</v>
       </c>
       <c r="F24" t="n">
         <v>5</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0.9699 ± 0.0002699</t>
+          <t>0.04811 ± 0.0001919</t>
         </is>
       </c>
     </row>
@@ -1181,21 +1181,21 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.96814523935318</v>
+        <v>0.0492212808790379</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0003577752986648186</v>
+        <v>0.000275921959119208</v>
       </c>
       <c r="F25" t="n">
         <v>5</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.9681 ± 0.0003578</t>
+          <t>0.04922 ± 0.0002759</t>
         </is>
       </c>
     </row>
@@ -1212,21 +1212,21 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>11.3538197647947</v>
+        <v>0.9673994421958924</v>
       </c>
       <c r="E26" t="n">
-        <v>0.06951382789543305</v>
+        <v>0.0003991396556738538</v>
       </c>
       <c r="F26" t="n">
         <v>5</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>11.35 ± 0.06951</t>
+          <t>0.9674 ± 0.0003991</t>
         </is>
       </c>
     </row>
@@ -1243,21 +1243,21 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>11.07042617840203</v>
+        <v>0.9690066933631897</v>
       </c>
       <c r="E27" t="n">
-        <v>0.06329615021594281</v>
+        <v>0.0003546163641341093</v>
       </c>
       <c r="F27" t="n">
         <v>5</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>11.07 ± 0.0633</t>
+          <t>0.969 ± 0.0003546</t>
         </is>
       </c>
     </row>
@@ -1274,21 +1274,21 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>11.05163647657597</v>
+        <v>0.9691120862960816</v>
       </c>
       <c r="E28" t="n">
-        <v>0.05200611919147764</v>
+        <v>0.0002913077525296171</v>
       </c>
       <c r="F28" t="n">
         <v>5</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>11.05 ± 0.05201</t>
+          <t>0.9691 ± 0.0002913</t>
         </is>
       </c>
     </row>
@@ -1305,21 +1305,21 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>11.12332375507181</v>
+        <v>0.9687103509902955</v>
       </c>
       <c r="E29" t="n">
-        <v>0.03544692699508916</v>
+        <v>0.0001997038942132785</v>
       </c>
       <c r="F29" t="n">
         <v>5</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>11.12 ± 0.03545</t>
+          <t>0.9687 ± 0.0001997</t>
         </is>
       </c>
     </row>
@@ -1336,50 +1336,360 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10.91687610069049</v>
+        <v>0.9697226881980896</v>
       </c>
       <c r="E30" t="n">
-        <v>0.04885675441896008</v>
+        <v>0.0003926035134185611</v>
       </c>
       <c r="F30" t="n">
         <v>5</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>10.92 ± 0.04886</t>
+          <t>0.9697 ± 0.0003926</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>proposed_no_fa</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.9694504380226135</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.0003472485642229245</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0.9695 ± 0.0003472</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>proposed_no_fusion</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.9695720314979553</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.0002425774034813482</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0.9696 ± 0.0002426</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>proposed_no_ta</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>horizon_15</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0.96814523935318</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.0003577752986648186</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0.9681 ± 0.0003578</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cnn</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>rmse</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D34" t="n">
+        <v>11.3538197647947</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.06951382789543305</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>11.35 ± 0.06951</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>11.07042617840203</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.06329615021594281</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>11.07 ± 0.0633</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>dcnn_rbilstm</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>11.05163647657597</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.05200611919147764</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>11.05 ± 0.05201</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>lstm</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>11.12332375507181</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.03544692699508916</v>
+      </c>
+      <c r="F37" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>11.12 ± 0.03545</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>10.94176527600902</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.07092130697487677</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>10.94 ± 0.07092</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>proposed_no_fa</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>10.99089366699856</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.0623783420290455</v>
+      </c>
+      <c r="F39" t="n">
+        <v>5</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>10.99 ± 0.06238</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>proposed_no_fusion</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>10.96906628386592</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.04375466353088314</v>
+      </c>
+      <c r="F40" t="n">
+        <v>5</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>10.97 ± 0.04375</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>proposed_no_ta</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
         <v>11.22322713139151</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E41" t="n">
         <v>0.06291455164167087</v>
       </c>
-      <c r="F31" t="n">
-        <v>5</v>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="F41" t="n">
+        <v>5</v>
+      </c>
+      <c r="G41" t="inlineStr">
         <is>
           <t>11.22 ± 0.06291</t>
         </is>
@@ -1448,16 +1758,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>18.02857142857142</v>
+        <v>28.33333333333334</v>
       </c>
       <c r="D2" t="n">
-        <v>0.002910808981707902</v>
+        <v>0.0001913128745172794</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G2" t="n">
         <v>5</v>
@@ -1475,16 +1785,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>23.85714285714286</v>
+        <v>28.66666666666666</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0002312745432846364</v>
+        <v>0.0001663985656509976</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G3" t="n">
         <v>5</v>
@@ -1502,16 +1812,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22.48571428571428</v>
+        <v>29.93333333333334</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0004231908480764213</v>
+        <v>9.767090528983251e-05</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
         <v>5</v>
@@ -1529,16 +1839,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.48571428571428</v>
+        <v>29.93333333333334</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0004231908480764213</v>
+        <v>9.767090528983251e-05</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
         <v>5</v>
@@ -1556,16 +1866,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22.48571428571428</v>
+        <v>29.93333333333334</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0004231908480764213</v>
+        <v>9.767090528983251e-05</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G6" t="n">
         <v>5</v>
@@ -1582,7 +1892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1620,11 +1930,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>proposed_no_fa</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3">
@@ -1640,11 +1950,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3.4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1660,11 +1970,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed_no_fusion</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="5">
@@ -1680,11 +1990,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="6">
@@ -1700,11 +2010,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="7">
@@ -1720,11 +2030,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="8">
@@ -1735,16 +2045,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>mape</t>
+          <t>mae</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="9">
@@ -1755,7 +2065,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>mape</t>
+          <t>mae</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1764,7 +2074,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1780,11 +2090,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed_no_fusion</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2.6</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="11">
@@ -1800,11 +2110,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed_no_fa</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="12">
@@ -1820,11 +2130,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>proposed_no_ta</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5.2</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="13">
@@ -1840,11 +2150,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>cnn</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="14">
@@ -1855,16 +2165,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="15">
@@ -1875,16 +2185,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="16">
@@ -1895,16 +2205,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2.8</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="17">
@@ -1915,7 +2225,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>nrmse</t>
+          <t>mape</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1924,7 +2234,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.4</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="18">
@@ -1940,11 +2250,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="19">
@@ -1960,11 +2270,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>cnn</t>
+          <t>proposed_no_fusion</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="20">
@@ -1975,16 +2285,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>proposed_no_fa</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="21">
@@ -1995,7 +2305,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2004,7 +2314,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2.8</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="22">
@@ -2015,7 +2325,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2024,7 +2334,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2.8</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="23">
@@ -2035,7 +2345,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2044,7 +2354,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3.4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="24">
@@ -2055,7 +2365,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2064,7 +2374,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -2075,7 +2385,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>nrmse</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2084,7 +2394,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
@@ -2095,7 +2405,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2104,7 +2414,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="27">
@@ -2115,16 +2425,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>cnn_lstm</t>
+          <t>proposed_no_fusion</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="28">
@@ -2135,12 +2445,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>dcnn_rbilstm</t>
+          <t>proposed_no_fa</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2155,16 +2465,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>cnn_lstm</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="30">
@@ -2175,16 +2485,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>rmse</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>proposed_no_ta</t>
+          <t>dcnn_rbilstm</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="31">
@@ -2195,16 +2505,216 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>lstm</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>proposed_no_ta</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>cnn</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>rmse</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>proposed_no_fusion</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>proposed_no_fa</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>dcnn_rbilstm</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>lstm</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>proposed_no_ta</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>horizon_15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>cnn</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>6</v>
+      <c r="D41" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>